<commit_message>
Add Sept'26 tracker column, retry Bunny Shield blocks, backfill Aug/Sept prices
Tracker's month columns stopped at Aug'26 so this month's scrapes were
silently skipping every row; added Sept'26 (via Excel so the Quarterly/
Delta-Monthly cross-sheet formulas shifted correctly) and backfilled the
now-closed August average, September month-to-date average, and current
price for all 24 items from bigmint.co's price-graph API, since the last
real update predates end of August.

fetch_prices() now retries with backoff when Bunny Shield's JS-only
challenge blocks a request instead of failing the item outright, and the
scrape loop paces requests instead of firing all 24 back-to-back, since
that burst pattern is what was tripping the shield mid-run.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01187aYocwEFakpDiNEoK3HW
</commit_message>
<xml_diff>
--- a/server/data/tracker.xlsx
+++ b/server/data/tracker.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="5760" yWindow="3456" windowWidth="17280" windowHeight="8784" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly" sheetId="1" state="visible" r:id="rId1"/>
@@ -1379,7 +1379,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1441,7 +1441,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1479,7 +1479,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -2060,7 +2060,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -2122,7 +2122,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -2160,7 +2160,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -2741,7 +2741,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -2803,7 +2803,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -2841,7 +2841,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -3422,7 +3422,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -3484,7 +3484,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -3522,7 +3522,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -4097,7 +4097,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -4159,7 +4159,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -4197,7 +4197,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -4778,7 +4778,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -4840,7 +4840,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -4878,7 +4878,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t>None</a:t>
+            <a:t/>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -5394,7 +5394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM25"/>
+  <dimension ref="A1:AN25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.6"/>
   <cols>
     <col width="51.5546875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5403,12 +5403,12 @@
     <col width="8.33203125" customWidth="1" min="4" max="16"/>
     <col width="10.21875" customWidth="1" min="17" max="21"/>
     <col width="10.21875" customWidth="1" style="12" min="22" max="26"/>
-    <col width="9.5546875" customWidth="1" style="72" min="27" max="33"/>
-    <col width="14.21875" customWidth="1" style="72" min="34" max="34"/>
-    <col width="69.21875" bestFit="1" customWidth="1" style="10" min="35" max="35"/>
-    <col width="78.5546875" bestFit="1" customWidth="1" min="36" max="36"/>
-    <col hidden="1" width="43.33203125" customWidth="1" min="37" max="38"/>
-    <col width="10.6640625" bestFit="1" customWidth="1" min="39" max="39"/>
+    <col width="9.5546875" customWidth="1" style="72" min="27" max="34"/>
+    <col width="14.21875" customWidth="1" style="72" min="35" max="35"/>
+    <col width="69.21875" bestFit="1" customWidth="1" style="10" min="36" max="36"/>
+    <col width="78.5546875" bestFit="1" customWidth="1" min="37" max="37"/>
+    <col hidden="1" width="43.33203125" customWidth="1" min="38" max="39"/>
+    <col width="10.6640625" bestFit="1" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1" ht="48" customFormat="1" customHeight="1" s="39">
@@ -5573,32 +5573,37 @@
           <t>Aug'26</t>
         </is>
       </c>
-      <c r="AH1" s="73" t="inlineStr">
+      <c r="AH1" s="36" t="inlineStr">
+        <is>
+          <t>Sept'26</t>
+        </is>
+      </c>
+      <c r="AI1" s="73" t="inlineStr">
         <is>
           <t xml:space="preserve">Current </t>
         </is>
       </c>
-      <c r="AI1" s="38" t="inlineStr">
+      <c r="AJ1" s="38" t="inlineStr">
         <is>
           <t>Link (Monthly Average)</t>
         </is>
       </c>
-      <c r="AJ1" s="34" t="inlineStr">
+      <c r="AK1" s="34" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="AK1" s="34" t="inlineStr">
+      <c r="AL1" s="34" t="inlineStr">
         <is>
           <t>Link (T-1 Prices)</t>
         </is>
       </c>
-      <c r="AL1" s="34" t="inlineStr">
+      <c r="AM1" s="34" t="inlineStr">
         <is>
           <t>Link (Monthly Average)</t>
         </is>
       </c>
-      <c r="AM1" s="38" t="n"/>
+      <c r="AN1" s="38" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -5702,27 +5707,30 @@
         <v>38205.77</v>
       </c>
       <c r="AG2" s="4" t="n">
-        <v>38900</v>
+        <v>38981.25</v>
       </c>
       <c r="AH2" s="4" t="n">
-        <v>38900</v>
-      </c>
-      <c r="AI2" s="6" t="inlineStr">
+        <v>40275</v>
+      </c>
+      <c r="AI2" s="4" t="n">
+        <v>40400</v>
+      </c>
+      <c r="AJ2" s="6" t="inlineStr">
         <is>
           <t>Pig Iron, DAP-Raipur, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ2" s="7" t="inlineStr">
+      <c r="AK2" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/pig-iron-dap-raipur-india-1102-f-INR</t>
         </is>
       </c>
-      <c r="AK2" s="7" t="inlineStr">
+      <c r="AL2" s="7" t="inlineStr">
         <is>
           <t>Pig Iron Prices – Daily Market Rates &amp; Trends | BigMint</t>
         </is>
       </c>
-      <c r="AL2" s="7" t="inlineStr">
+      <c r="AM2" s="7" t="inlineStr">
         <is>
           <t>Pig Iron, DAP-Raipur, India | BigMint</t>
         </is>
@@ -5830,27 +5838,30 @@
         <v>40644.23</v>
       </c>
       <c r="AG3" s="4" t="n">
-        <v>40900</v>
+        <v>41072.92</v>
       </c>
       <c r="AH3" s="4" t="n">
-        <v>40900</v>
-      </c>
-      <c r="AI3" s="8" t="inlineStr">
+        <v>42072.73</v>
+      </c>
+      <c r="AI3" s="4" t="n">
+        <v>42400</v>
+      </c>
+      <c r="AJ3" s="8" t="inlineStr">
         <is>
           <t>Pig Iron, DAP-Ludhiana, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ3" s="7" t="inlineStr">
+      <c r="AK3" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/pig-iron-dap-ludhiana-india-1100-f-INR</t>
         </is>
       </c>
-      <c r="AK3" s="7" t="inlineStr">
+      <c r="AL3" s="7" t="inlineStr">
         <is>
           <t>Pig Iron Prices – Daily Market Rates &amp; Trends | BigMint</t>
         </is>
       </c>
-      <c r="AL3" s="7" t="inlineStr">
+      <c r="AM3" s="7" t="inlineStr">
         <is>
           <t>Pig Iron, DAP-Ludhiana, India | BigMint</t>
         </is>
@@ -5958,27 +5969,30 @@
         <v>37819.23</v>
       </c>
       <c r="AG4" s="4" t="n">
-        <v>38550</v>
+        <v>38660.42</v>
       </c>
       <c r="AH4" s="4" t="n">
-        <v>38550</v>
-      </c>
-      <c r="AI4" s="6" t="inlineStr">
+        <v>40263.64</v>
+      </c>
+      <c r="AI4" s="4" t="n">
+        <v>41550</v>
+      </c>
+      <c r="AJ4" s="6" t="inlineStr">
         <is>
           <t>Pig Iron, Exw-Durgapur, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ4" s="7" t="inlineStr">
+      <c r="AK4" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/pig-iron-exw-durgapur-india-1096-f-INR</t>
         </is>
       </c>
-      <c r="AK4" s="7" t="inlineStr">
+      <c r="AL4" s="7" t="inlineStr">
         <is>
           <t>Pig Iron Prices – Daily Market Rates &amp; Trends | BigMint</t>
         </is>
       </c>
-      <c r="AL4" s="7" t="inlineStr">
+      <c r="AM4" s="7" t="inlineStr">
         <is>
           <t>Pig Iron, Exw-Durgapur, India | BigMint</t>
         </is>
@@ -6086,27 +6100,30 @@
         <v>37442.31</v>
       </c>
       <c r="AG5" s="4" t="n">
-        <v>39200</v>
+        <v>38862.5</v>
       </c>
       <c r="AH5" s="4" t="n">
-        <v>39200</v>
-      </c>
-      <c r="AI5" s="8" t="inlineStr">
+        <v>40236.36</v>
+      </c>
+      <c r="AI5" s="4" t="n">
+        <v>41000</v>
+      </c>
+      <c r="AJ5" s="8" t="inlineStr">
         <is>
           <t>Pig Iron, DAP-Hyderabad, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ5" s="7" t="inlineStr">
+      <c r="AK5" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/pig-iron-dap-hyderabad-india-1098-f-INR</t>
         </is>
       </c>
-      <c r="AK5" s="7" t="inlineStr">
+      <c r="AL5" s="7" t="inlineStr">
         <is>
           <t>Pig Iron Prices – Daily Market Rates &amp; Trends | BigMint</t>
         </is>
       </c>
-      <c r="AL5" s="7" t="inlineStr">
+      <c r="AM5" s="7" t="inlineStr">
         <is>
           <t>Pig Iron, DAP-Hyderabad, India | BigMint</t>
         </is>
@@ -6214,27 +6231,30 @@
         <v>45592.31</v>
       </c>
       <c r="AG6" s="4" t="n">
-        <v>47700</v>
+        <v>47266.67</v>
       </c>
       <c r="AH6" s="4" t="n">
-        <v>47700</v>
-      </c>
-      <c r="AI6" s="9" t="inlineStr">
+        <v>47181.82</v>
+      </c>
+      <c r="AI6" s="4" t="n">
+        <v>47000</v>
+      </c>
+      <c r="AJ6" s="9" t="inlineStr">
         <is>
           <t>Pig Iron, DAP-Ludhiana, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ6" s="7" t="inlineStr">
+      <c r="AK6" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/pig-iron-dap-ludhiana-india-1108-f-INR</t>
         </is>
       </c>
-      <c r="AK6" s="7" t="inlineStr">
+      <c r="AL6" s="7" t="inlineStr">
         <is>
           <t>Pig Iron Prices – Daily Market Rates &amp; Trends | BigMint</t>
         </is>
       </c>
-      <c r="AL6" s="7" t="inlineStr">
+      <c r="AM6" s="7" t="inlineStr">
         <is>
           <t>Pig Iron, DAP-Ludhiana, India | BigMint</t>
         </is>
@@ -6344,27 +6364,30 @@
         <v>43000</v>
       </c>
       <c r="AG7" s="4" t="n">
-        <v>45000</v>
+        <v>44208.33</v>
       </c>
       <c r="AH7" s="4" t="n">
         <v>45000</v>
       </c>
-      <c r="AI7" s="30" t="inlineStr">
+      <c r="AI7" s="4" t="n">
+        <v>45000</v>
+      </c>
+      <c r="AJ7" s="30" t="inlineStr">
         <is>
           <t>Pig Iron, Exw-Durgapur, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ7" s="7" t="inlineStr">
+      <c r="AK7" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/pig-iron-exw-durgapur-india-1105-f-INR</t>
         </is>
       </c>
-      <c r="AK7" s="7" t="inlineStr">
+      <c r="AL7" s="7" t="inlineStr">
         <is>
           <t>Pig Iron Prices – Daily Market Rates &amp; Trends | BigMint</t>
         </is>
       </c>
-      <c r="AL7" s="7" t="inlineStr">
+      <c r="AM7" s="7" t="inlineStr">
         <is>
           <t>Pig Iron, Exw-Durgapur, India | BigMint</t>
         </is>
@@ -6472,27 +6495,30 @@
         <v>36375</v>
       </c>
       <c r="AG8" s="4" t="n">
-        <v>37100</v>
+        <v>37002.08</v>
       </c>
       <c r="AH8" s="4" t="n">
-        <v>37100</v>
-      </c>
-      <c r="AI8" s="9" t="inlineStr">
+        <v>38336.36</v>
+      </c>
+      <c r="AI8" s="4" t="n">
+        <v>39000</v>
+      </c>
+      <c r="AJ8" s="9" t="inlineStr">
         <is>
           <t>Melting Scrap, DAP-Raipur, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ8" s="7" t="inlineStr">
+      <c r="AK8" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/melting-scrap-dap-raipur-india-1040-f-INR</t>
         </is>
       </c>
-      <c r="AK8" s="7" t="inlineStr">
+      <c r="AL8" s="7" t="inlineStr">
         <is>
           <t>Melting Scrap Prices – Live Market Updates | BigMint</t>
         </is>
       </c>
-      <c r="AL8" s="7" t="inlineStr">
+      <c r="AM8" s="7" t="inlineStr">
         <is>
           <t>Melting Scrap, DAP-Raipur, India | BigMint</t>
         </is>
@@ -6600,27 +6626,30 @@
         <v>34161.54</v>
       </c>
       <c r="AG9" s="4" t="n">
-        <v>34550</v>
+        <v>34693.75</v>
       </c>
       <c r="AH9" s="4" t="n">
-        <v>34550</v>
-      </c>
-      <c r="AI9" s="9" t="inlineStr">
+        <v>36377.27</v>
+      </c>
+      <c r="AI9" s="4" t="n">
+        <v>36800</v>
+      </c>
+      <c r="AJ9" s="9" t="inlineStr">
         <is>
           <t>Melting Scrap, DAP-Raipur, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ9" s="7" t="inlineStr">
+      <c r="AK9" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/melting-scrap-dap-raipur-india-1041-f-INR</t>
         </is>
       </c>
-      <c r="AK9" s="7" t="inlineStr">
+      <c r="AL9" s="7" t="inlineStr">
         <is>
           <t>Melting Scrap Prices – Live Market Updates | BigMint</t>
         </is>
       </c>
-      <c r="AL9" s="7" t="inlineStr">
+      <c r="AM9" s="7" t="inlineStr">
         <is>
           <t>Melting Scrap, DAP-Raipur, India | BigMint</t>
         </is>
@@ -6728,27 +6757,30 @@
         <v>23915.38</v>
       </c>
       <c r="AG10" s="4" t="n">
-        <v>27900</v>
+        <v>26812.5</v>
       </c>
       <c r="AH10" s="4" t="n">
-        <v>27900</v>
-      </c>
-      <c r="AI10" s="9" t="inlineStr">
+        <v>29031.82</v>
+      </c>
+      <c r="AI10" s="4" t="n">
+        <v>29650</v>
+      </c>
+      <c r="AJ10" s="9" t="inlineStr">
         <is>
           <t>Sponge Iron, PDRI, Exw-Raipur, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ10" s="7" t="inlineStr">
+      <c r="AK10" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/sponge-iron-pdri-exw-raipur-india-1091-f-INR</t>
         </is>
       </c>
-      <c r="AK10" s="7" t="inlineStr">
+      <c r="AL10" s="7" t="inlineStr">
         <is>
           <t>Sponge Iron Prices – Daily Market Rates | BigMint</t>
         </is>
       </c>
-      <c r="AL10" s="7" t="inlineStr">
+      <c r="AM10" s="7" t="inlineStr">
         <is>
           <t>Sponge Iron, PDRI, Exw-Raipur, India | BigMint</t>
         </is>
@@ -6856,27 +6888,30 @@
         <v>43907.69</v>
       </c>
       <c r="AG11" s="4" t="n">
-        <v>47900</v>
+        <v>47237.5</v>
       </c>
       <c r="AH11" s="4" t="n">
-        <v>47900</v>
-      </c>
-      <c r="AI11" s="9" t="inlineStr">
+        <v>50181.82</v>
+      </c>
+      <c r="AI11" s="4" t="n">
+        <v>51400</v>
+      </c>
+      <c r="AJ11" s="9" t="inlineStr">
         <is>
           <t>Rebar, Exw-Mumbai, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ11" s="7" t="inlineStr">
+      <c r="AK11" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/rebar-exw-mumbai-india-1122-f-INR</t>
         </is>
       </c>
-      <c r="AK11" s="7" t="inlineStr">
+      <c r="AL11" s="7" t="inlineStr">
         <is>
           <t>Rebar Prices – Daily Steel TMT &amp; Rebar Market Rates | BigMint</t>
         </is>
       </c>
-      <c r="AL11" s="7" t="inlineStr">
+      <c r="AM11" s="7" t="inlineStr">
         <is>
           <t>Rebar, Exw-Mumbai, India | BigMint</t>
         </is>
@@ -6984,27 +7019,30 @@
         <v>40100</v>
       </c>
       <c r="AG12" s="4" t="n">
-        <v>42600</v>
+        <v>41733.33</v>
       </c>
       <c r="AH12" s="4" t="n">
-        <v>42600</v>
-      </c>
-      <c r="AI12" s="9" t="inlineStr">
+        <v>44772.73</v>
+      </c>
+      <c r="AI12" s="4" t="n">
+        <v>46500</v>
+      </c>
+      <c r="AJ12" s="9" t="inlineStr">
         <is>
           <t>Rebar, Exw-Raipur, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ12" s="7" t="inlineStr">
+      <c r="AK12" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/rebar-exw-raipur-india-1117-f-INR</t>
         </is>
       </c>
-      <c r="AK12" s="7" t="inlineStr">
+      <c r="AL12" s="7" t="inlineStr">
         <is>
           <t>Rebar Prices – Daily Steel TMT &amp; Rebar Market Rates | BigMint</t>
         </is>
       </c>
-      <c r="AL12" s="7" t="inlineStr">
+      <c r="AM12" s="7" t="inlineStr">
         <is>
           <t>Rebar, Exw-Raipur, India | BigMint</t>
         </is>
@@ -7112,27 +7150,30 @@
         <v>49077.78</v>
       </c>
       <c r="AG13" s="4" t="n">
-        <v>53900</v>
+        <v>53293.75</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>53900</v>
-      </c>
-      <c r="AI13" s="9" t="inlineStr">
+        <v>57575</v>
+      </c>
+      <c r="AI13" s="4" t="n">
+        <v>58150</v>
+      </c>
+      <c r="AJ13" s="9" t="inlineStr">
         <is>
           <t>Rebar, Exy-Mumbai, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ13" s="7" t="inlineStr">
+      <c r="AK13" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/rebar-exy-mumbai-india-1127-f-INR</t>
         </is>
       </c>
-      <c r="AK13" s="7" t="inlineStr">
+      <c r="AL13" s="7" t="inlineStr">
         <is>
           <t>Rebar Prices – Daily Steel TMT &amp; Rebar Market Rates | BigMint</t>
         </is>
       </c>
-      <c r="AL13" s="7" t="inlineStr">
+      <c r="AM13" s="7" t="inlineStr">
         <is>
           <t>Rebar, Exy-Mumbai, India | BigMint</t>
         </is>
@@ -7240,27 +7281,30 @@
         <v>38164.81</v>
       </c>
       <c r="AG14" s="4" t="n">
-        <v>40400</v>
+        <v>39650</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>40400</v>
-      </c>
-      <c r="AI14" s="9" t="inlineStr">
+        <v>42631.82</v>
+      </c>
+      <c r="AI14" s="4" t="n">
+        <v>44000</v>
+      </c>
+      <c r="AJ14" s="9" t="inlineStr">
         <is>
           <t>Billet Index, Exw-Raipur, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ14" s="7" t="inlineStr">
+      <c r="AK14" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/billet-index-exw-raipur-india-1067-f-INR</t>
         </is>
       </c>
-      <c r="AK14" s="7" t="inlineStr">
+      <c r="AL14" s="7" t="inlineStr">
         <is>
           <t>Billet, Bloom &amp; Ingot Prices – Steel Market Rates Today | BigMint</t>
         </is>
       </c>
-      <c r="AL14" s="7" t="inlineStr">
+      <c r="AM14" s="7" t="inlineStr">
         <is>
           <t>Billet Index, Exw-Raipur, India | BigMint</t>
         </is>
@@ -7368,27 +7412,30 @@
         <v>37824.07</v>
       </c>
       <c r="AG15" s="4" t="n">
-        <v>39950</v>
+        <v>39256.25</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>39950</v>
-      </c>
-      <c r="AI15" s="9" t="inlineStr">
+        <v>42168.18</v>
+      </c>
+      <c r="AI15" s="4" t="n">
+        <v>43500</v>
+      </c>
+      <c r="AJ15" s="9" t="inlineStr">
         <is>
           <t>Ingot, Exw-Raipur, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ15" s="7" t="inlineStr">
+      <c r="AK15" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/ingot-exw-raipur-india-1275-f-INR</t>
         </is>
       </c>
-      <c r="AK15" s="7" t="inlineStr">
+      <c r="AL15" s="7" t="inlineStr">
         <is>
           <t>Billet, Bloom &amp; Ingot Prices – Steel Market Rates Today | BigMint</t>
         </is>
       </c>
-      <c r="AL15" s="7" t="inlineStr">
+      <c r="AM15" s="7" t="inlineStr">
         <is>
           <t>Ingot, Exw-Raipur, India | BigMint</t>
         </is>
@@ -7496,27 +7543,30 @@
         <v>9683.33</v>
       </c>
       <c r="AG16" s="4" t="n">
-        <v>10600</v>
+        <v>10431.25</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>10600</v>
-      </c>
-      <c r="AI16" s="9" t="inlineStr">
+        <v>11000</v>
+      </c>
+      <c r="AI16" s="4" t="n">
+        <v>11000</v>
+      </c>
+      <c r="AJ16" s="9" t="inlineStr">
         <is>
           <t>Pellet Index, PELLEX, DAP-Raipur, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ16" s="7" t="inlineStr">
+      <c r="AK16" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/pellet-index-pellex-dap-raipur-india-1401-f-INR</t>
         </is>
       </c>
-      <c r="AK16" s="7" t="inlineStr">
+      <c r="AL16" s="7" t="inlineStr">
         <is>
           <t>Iron Ore Pellets Prices – Live Market Updates | BigMint</t>
         </is>
       </c>
-      <c r="AL16" s="7" t="inlineStr">
+      <c r="AM16" s="7" t="inlineStr">
         <is>
           <t>Pellet Index, PELLEX, DAP-Raipur, India | BigMint</t>
         </is>
@@ -7624,27 +7674,30 @@
         <v>57888.89</v>
       </c>
       <c r="AG17" s="4" t="n">
-        <v>58800</v>
+        <v>58575</v>
       </c>
       <c r="AH17" s="4" t="n">
-        <v>58800</v>
-      </c>
-      <c r="AI17" s="9" t="inlineStr">
+        <v>62100</v>
+      </c>
+      <c r="AI17" s="4" t="n">
+        <v>62200</v>
+      </c>
+      <c r="AJ17" s="9" t="inlineStr">
         <is>
           <t>HRC, Exy-Mumbai, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ17" s="7" t="inlineStr">
+      <c r="AK17" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/hrc-exy-mumbai-india-1234-f-INR</t>
         </is>
       </c>
-      <c r="AK17" s="7" t="inlineStr">
+      <c r="AL17" s="7" t="inlineStr">
         <is>
           <t>HRC Prices – Hot Rolled Coil Market Rates Today | BigMint</t>
         </is>
       </c>
-      <c r="AL17" s="7" t="inlineStr">
+      <c r="AM17" s="7" t="inlineStr">
         <is>
           <t>HRC, Exy-Mumbai, India | BigMint</t>
         </is>
@@ -7752,27 +7805,30 @@
         <v>64988.89</v>
       </c>
       <c r="AG18" s="4" t="n">
-        <v>65900</v>
+        <v>65725</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>65900</v>
-      </c>
-      <c r="AI18" s="9" t="inlineStr">
+        <v>71400</v>
+      </c>
+      <c r="AI18" s="4" t="n">
+        <v>72000</v>
+      </c>
+      <c r="AJ18" s="9" t="inlineStr">
         <is>
           <t>CRC, Exy-Mumbai, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ18" s="7" t="inlineStr">
+      <c r="AK18" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/crc-exy-mumbai-india-1243-f-INR</t>
         </is>
       </c>
-      <c r="AK18" s="7" t="inlineStr">
+      <c r="AL18" s="7" t="inlineStr">
         <is>
           <t>CRC Prices – Cold Rolled Coil Market Rates Today | BigMint</t>
         </is>
       </c>
-      <c r="AL18" s="7" t="inlineStr">
+      <c r="AM18" s="7" t="inlineStr">
         <is>
           <t>CRC, Exy-Mumbai, India | BigMint</t>
         </is>
@@ -7880,27 +7936,30 @@
         <v>60440</v>
       </c>
       <c r="AG19" s="4" t="n">
-        <v>61500</v>
+        <v>61450</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>61500</v>
-      </c>
-      <c r="AI19" s="9" t="inlineStr">
+        <v>63900</v>
+      </c>
+      <c r="AI19" s="4" t="n">
+        <v>63900</v>
+      </c>
+      <c r="AJ19" s="9" t="inlineStr">
         <is>
           <t>HR Plate, Exy-Mumbai, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ19" s="7" t="inlineStr">
+      <c r="AK19" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/hr-plate-exy-mumbai-india-1496-f-INR</t>
         </is>
       </c>
-      <c r="AK19" s="7" t="inlineStr">
+      <c r="AL19" s="7" t="inlineStr">
         <is>
           <t>HR Plate Prices – Hot Rolled Plate Market Rates Today | BigMint</t>
         </is>
       </c>
-      <c r="AL19" s="7" t="inlineStr">
+      <c r="AM19" s="7" t="inlineStr">
         <is>
           <t>HR Plate, Exy-Mumbai, India | BigMint</t>
         </is>
@@ -8008,27 +8067,30 @@
         <v>72380</v>
       </c>
       <c r="AG20" s="4" t="n">
-        <v>74200</v>
+        <v>74100</v>
       </c>
       <c r="AH20" s="4" t="n">
-        <v>74200</v>
-      </c>
-      <c r="AI20" s="10" t="inlineStr">
+        <v>77500</v>
+      </c>
+      <c r="AI20" s="4" t="n">
+        <v>78300</v>
+      </c>
+      <c r="AJ20" s="10" t="inlineStr">
         <is>
           <t>GP, Exy-Mumbai, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ20" s="7" t="inlineStr">
+      <c r="AK20" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/gp-exy-mumbai-india-1678-f-INR</t>
         </is>
       </c>
-      <c r="AK20" s="7" t="inlineStr">
+      <c r="AL20" s="7" t="inlineStr">
         <is>
           <t>Prices | BigMint</t>
         </is>
       </c>
-      <c r="AL20" s="7" t="inlineStr">
+      <c r="AM20" s="7" t="inlineStr">
         <is>
           <t>GP, Exy-Mumbai, India | BigMint</t>
         </is>
@@ -8136,27 +8198,30 @@
         <v>61380</v>
       </c>
       <c r="AG21" s="4" t="n">
-        <v>61700</v>
+        <v>61625</v>
       </c>
       <c r="AH21" s="4" t="n">
-        <v>61700</v>
-      </c>
-      <c r="AI21" s="10" t="inlineStr">
+        <v>64250</v>
+      </c>
+      <c r="AI21" s="4" t="n">
+        <v>64900</v>
+      </c>
+      <c r="AJ21" s="10" t="inlineStr">
         <is>
           <t>ERW Pipe (HR Coil based), Exy-Mumbai, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ21" s="7" t="inlineStr">
+      <c r="AK21" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/erw-pipe-hr-coil-based-exy-mumbai-india-1475-f-INR</t>
         </is>
       </c>
-      <c r="AK21" s="7" t="inlineStr">
+      <c r="AL21" s="7" t="inlineStr">
         <is>
           <t>Steel Pipes Prices – Market Rates for MS &amp; GI Pipes | BigMint</t>
         </is>
       </c>
-      <c r="AL21" s="7" t="inlineStr">
+      <c r="AM21" s="7" t="inlineStr">
         <is>
           <t>ERW Pipe (HR Coil based), Exy-Mumbai, India | BigMint</t>
         </is>
@@ -8264,27 +8329,30 @@
         <v>62080</v>
       </c>
       <c r="AG22" s="4" t="n">
-        <v>62400</v>
+        <v>62350</v>
       </c>
       <c r="AH22" s="4" t="n">
-        <v>62400</v>
-      </c>
-      <c r="AI22" s="9" t="inlineStr">
+        <v>63950</v>
+      </c>
+      <c r="AI22" s="4" t="n">
+        <v>64400</v>
+      </c>
+      <c r="AJ22" s="9" t="inlineStr">
         <is>
           <t>ERW Pipe (HR Coil based), Exy-Delhi, India | BigMint</t>
         </is>
       </c>
-      <c r="AJ22" s="7" t="inlineStr">
+      <c r="AK22" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/erw-pipe-hr-coil-based-exy-delhi-india-1426-f-INR</t>
         </is>
       </c>
-      <c r="AK22" s="7" t="inlineStr">
+      <c r="AL22" s="7" t="inlineStr">
         <is>
           <t>Steel Pipes Prices – Market Rates for MS &amp; GI Pipes | BigMint</t>
         </is>
       </c>
-      <c r="AL22" s="7" t="inlineStr">
+      <c r="AM22" s="7" t="inlineStr">
         <is>
           <t>ERW Pipe (HR Coil based), Exy-Delhi, India | BigMint</t>
         </is>
@@ -8386,12 +8454,15 @@
       <c r="AH23" s="4" t="n">
         <v>90000</v>
       </c>
-      <c r="AI23" s="9" t="inlineStr">
+      <c r="AI23" s="4" t="n">
+        <v>90000</v>
+      </c>
+      <c r="AJ23" s="9" t="inlineStr">
         <is>
           <t>Galvalume, Exy-Mumbai, India (0.5mm / CTL, 1220mm, AZ 150, IS15961)</t>
         </is>
       </c>
-      <c r="AJ23" s="7" t="inlineStr">
+      <c r="AK23" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/galvalume-exy-mumbai-india-1521-f-INR</t>
         </is>
@@ -8493,12 +8564,15 @@
       <c r="AH24" s="4" t="n">
         <v>87000</v>
       </c>
-      <c r="AI24" s="9" t="inlineStr">
+      <c r="AI24" s="4" t="n">
+        <v>87000</v>
+      </c>
+      <c r="AJ24" s="9" t="inlineStr">
         <is>
           <t>Galvalume, Exy-Mumbai, India (0.5mm / CTL, 1220mm, AZ 70, IS15961)</t>
         </is>
       </c>
-      <c r="AJ24" s="7" t="inlineStr">
+      <c r="AK24" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/galvalume-exy-mumbai-india-1518-f-INR</t>
         </is>
@@ -8619,17 +8693,20 @@
         <v>84800</v>
       </c>
       <c r="AG25" s="4" t="n">
-        <v>85300</v>
+        <v>85450</v>
       </c>
       <c r="AH25" s="4" t="n">
-        <v>85300</v>
-      </c>
-      <c r="AI25" s="9" t="inlineStr">
+        <v>87150</v>
+      </c>
+      <c r="AI25" s="4" t="n">
+        <v>87300</v>
+      </c>
+      <c r="AJ25" s="9" t="inlineStr">
         <is>
           <t>PPGI, Exy-Mumbai, India (0.5mm / CTL, 90 GSM, IS14246)</t>
         </is>
       </c>
-      <c r="AJ25" s="7" t="inlineStr">
+      <c r="AK25" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/ppgi-exy-mumbai-india-1369-f-INR</t>
         </is>
@@ -8639,112 +8716,112 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/pig-iron" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" display="https://www.bigmint.co/prices/detail/pig-iron-dap-raipur-india-1102-f-INR" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK2" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/pig-iron" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL2" display="https://www.bigmint.co/prices/detail/pig-iron-dap-raipur-india-1102-f-INR" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL2" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/pig-iron" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM2" display="https://www.bigmint.co/prices/detail/pig-iron-dap-raipur-india-1102-f-INR" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/pig-iron" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" display="https://www.bigmint.co/prices/detail/pig-iron-dap-ludhiana-india-1100-f-INR" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ3" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK3" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/pig-iron" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL3" display="https://www.bigmint.co/prices/detail/pig-iron-dap-ludhiana-india-1100-f-INR" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL3" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/pig-iron" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM3" display="https://www.bigmint.co/prices/detail/pig-iron-dap-ludhiana-india-1100-f-INR" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/pig-iron" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" display="https://www.bigmint.co/prices/detail/pig-iron-exw-durgapur-india-1096-f-INR" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ4" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK4" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/pig-iron" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL4" display="https://www.bigmint.co/prices/detail/pig-iron-exw-durgapur-india-1096-f-INR" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK4" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL4" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/pig-iron" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM4" display="https://www.bigmint.co/prices/detail/pig-iron-exw-durgapur-india-1096-f-INR" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/pig-iron" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" display="https://www.bigmint.co/prices/detail/pig-iron-dap-hyderabad-india-1098-f-INR" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ5" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK5" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/pig-iron" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL5" display="https://www.bigmint.co/prices/detail/pig-iron-dap-hyderabad-india-1098-f-INR" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK5" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL5" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/pig-iron" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM5" display="https://www.bigmint.co/prices/detail/pig-iron-dap-hyderabad-india-1098-f-INR" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/pig-iron" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" display="https://www.bigmint.co/prices/detail/pig-iron-dap-ludhiana-india-1108-f-INR" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ6" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK6" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/pig-iron" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL6" display="https://www.bigmint.co/prices/detail/pig-iron-dap-ludhiana-india-1108-f-INR" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK6" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL6" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/pig-iron" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM6" display="https://www.bigmint.co/prices/detail/pig-iron-dap-ludhiana-india-1108-f-INR" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/pig-iron" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" display="https://www.bigmint.co/prices/detail/pig-iron-exw-durgapur-india-1105-f-INR" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ7" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK7" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/pig-iron" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL7" display="https://www.bigmint.co/prices/detail/pig-iron-exw-durgapur-india-1105-f-INR" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK7" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL7" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/pig-iron" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM7" display="https://www.bigmint.co/prices/detail/pig-iron-exw-durgapur-india-1105-f-INR" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/melting-scrap" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" display="https://www.bigmint.co/prices/detail/melting-scrap-dap-raipur-india-1040-f-INR" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ8" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK8" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/melting-scrap" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL8" display="https://www.bigmint.co/prices/detail/melting-scrap-dap-raipur-india-1040-f-INR" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK8" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL8" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/melting-scrap" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM8" display="https://www.bigmint.co/prices/detail/melting-scrap-dap-raipur-india-1040-f-INR" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/melting-scrap" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" display="https://www.bigmint.co/prices/detail/melting-scrap-dap-raipur-india-1041-f-INR" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ9" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK9" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/melting-scrap" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL9" display="https://www.bigmint.co/prices/detail/melting-scrap-dap-raipur-india-1041-f-INR" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK9" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL9" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/melting-scrap" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM9" display="https://www.bigmint.co/prices/detail/melting-scrap-dap-raipur-india-1041-f-INR" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/sponge-iron" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" display="https://www.bigmint.co/prices/detail/sponge-iron-pdri-exw-raipur-india-1091-f-INR" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ10" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK10" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/sponge-iron" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL10" display="https://www.bigmint.co/prices/detail/sponge-iron-pdri-exw-raipur-india-1091-f-INR" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK10" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL10" display="https://www.bigmint.co/prices/ferrous/scrap-metallics/sponge-iron" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM10" display="https://www.bigmint.co/prices/detail/sponge-iron-pdri-exw-raipur-india-1091-f-INR" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" display="https://www.bigmint.co/prices/ferrous/steel/rebar" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" display="https://www.bigmint.co/prices/detail/rebar-exw-mumbai-india-1122-f-INR" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ11" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK11" display="https://www.bigmint.co/prices/ferrous/steel/rebar" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL11" display="https://www.bigmint.co/prices/detail/rebar-exw-mumbai-india-1122-f-INR" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK11" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL11" display="https://www.bigmint.co/prices/ferrous/steel/rebar" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM11" display="https://www.bigmint.co/prices/detail/rebar-exw-mumbai-india-1122-f-INR" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" display="https://www.bigmint.co/prices/ferrous/steel/rebar" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" display="https://www.bigmint.co/prices/detail/rebar-exw-raipur-india-1117-f-INR" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ12" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK12" display="https://www.bigmint.co/prices/ferrous/steel/rebar" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL12" display="https://www.bigmint.co/prices/detail/rebar-exw-raipur-india-1117-f-INR" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK12" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL12" display="https://www.bigmint.co/prices/ferrous/steel/rebar" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM12" display="https://www.bigmint.co/prices/detail/rebar-exw-raipur-india-1117-f-INR" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" display="https://www.bigmint.co/prices/ferrous/steel/rebar" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" display="https://www.bigmint.co/prices/detail/rebar-exy-mumbai-india-1127-f-INR" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ13" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK13" display="https://www.bigmint.co/prices/ferrous/steel/rebar" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL13" display="https://www.bigmint.co/prices/detail/rebar-exy-mumbai-india-1127-f-INR" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK13" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL13" display="https://www.bigmint.co/prices/ferrous/steel/rebar" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM13" display="https://www.bigmint.co/prices/detail/rebar-exy-mumbai-india-1127-f-INR" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" display="https://www.bigmint.co/prices/ferrous/steel/billetbloomingot" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" display="https://www.bigmint.co/prices/detail/billet-index-exw-raipur-india-1067-f-INR" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ14" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK14" display="https://www.bigmint.co/prices/ferrous/steel/billetbloomingot" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL14" display="https://www.bigmint.co/prices/detail/billet-index-exw-raipur-india-1067-f-INR" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK14" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL14" display="https://www.bigmint.co/prices/ferrous/steel/billetbloomingot" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM14" display="https://www.bigmint.co/prices/detail/billet-index-exw-raipur-india-1067-f-INR" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" display="https://www.bigmint.co/prices/ferrous/steel/billetbloomingot" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" display="https://www.bigmint.co/prices/detail/ingot-exw-raipur-india-1275-f-INR" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ15" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK15" display="https://www.bigmint.co/prices/ferrous/steel/billetbloomingot" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL15" display="https://www.bigmint.co/prices/detail/ingot-exw-raipur-india-1275-f-INR" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK15" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL15" display="https://www.bigmint.co/prices/ferrous/steel/billetbloomingot" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM15" display="https://www.bigmint.co/prices/detail/ingot-exw-raipur-india-1275-f-INR" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" display="https://www.bigmint.co/prices/ferrous/iron-ore/pellets" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" display="https://www.bigmint.co/prices/detail/pellet-index-pellex-dap-raipur-india-1401-f-INR" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ16" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK16" display="https://www.bigmint.co/prices/ferrous/iron-ore/pellets" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL16" display="https://www.bigmint.co/prices/detail/pellet-index-pellex-dap-raipur-india-1401-f-INR" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK16" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL16" display="https://www.bigmint.co/prices/ferrous/iron-ore/pellets" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM16" display="https://www.bigmint.co/prices/detail/pellet-index-pellex-dap-raipur-india-1401-f-INR" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" display="https://www.bigmint.co/prices/ferrous/steel/hrc" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" display="https://www.bigmint.co/prices/detail/hrc-exy-mumbai-india-1234-f-INR" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ17" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK17" display="https://www.bigmint.co/prices/ferrous/steel/hrc" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL17" display="https://www.bigmint.co/prices/detail/hrc-exy-mumbai-india-1234-f-INR" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK17" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL17" display="https://www.bigmint.co/prices/ferrous/steel/hrc" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM17" display="https://www.bigmint.co/prices/detail/hrc-exy-mumbai-india-1234-f-INR" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" display="https://www.bigmint.co/prices/ferrous/steel/crc" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" display="https://www.bigmint.co/prices/detail/crc-exy-mumbai-india-1243-f-INR" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ18" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK18" display="https://www.bigmint.co/prices/ferrous/steel/crc" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL18" display="https://www.bigmint.co/prices/detail/crc-exy-mumbai-india-1243-f-INR" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK18" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL18" display="https://www.bigmint.co/prices/ferrous/steel/crc" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM18" display="https://www.bigmint.co/prices/detail/crc-exy-mumbai-india-1243-f-INR" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" display="https://www.bigmint.co/prices/ferrous/steel/hr-plate" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" display="https://www.bigmint.co/prices/detail/hr-plate-exy-mumbai-india-1496-f-INR" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ19" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK19" display="https://www.bigmint.co/prices/ferrous/steel/hr-plate" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL19" display="https://www.bigmint.co/prices/detail/hr-plate-exy-mumbai-india-1496-f-INR" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK19" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL19" display="https://www.bigmint.co/prices/ferrous/steel/hr-plate" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM19" display="https://www.bigmint.co/prices/detail/hr-plate-exy-mumbai-india-1496-f-INR" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" display="https://www.bigmint.co/prices/ferrous/steel/gp" r:id="rId91"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" display="https://www.bigmint.co/prices/detail/gp-exy-mumbai-india-1678-f-INR" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ20" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK20" display="https://www.bigmint.co/prices/ferrous/steel/gp" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL20" display="https://www.bigmint.co/prices/detail/gp-exy-mumbai-india-1678-f-INR" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK20" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL20" display="https://www.bigmint.co/prices/ferrous/steel/gp" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM20" display="https://www.bigmint.co/prices/detail/gp-exy-mumbai-india-1678-f-INR" r:id="rId95"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" display="https://www.bigmint.co/prices/ferrous/steel/pipes" r:id="rId96"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" display="https://www.bigmint.co/prices/detail/erw-pipe-hr-coil-based-exy-mumbai-india-1475-f-INR" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ21" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK21" display="https://www.bigmint.co/prices/ferrous/steel/pipes" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL21" display="https://www.bigmint.co/prices/detail/erw-pipe-hr-coil-based-exy-mumbai-india-1475-f-INR" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK21" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL21" display="https://www.bigmint.co/prices/ferrous/steel/pipes" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM21" display="https://www.bigmint.co/prices/detail/erw-pipe-hr-coil-based-exy-mumbai-india-1475-f-INR" r:id="rId100"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" display="https://www.bigmint.co/prices/ferrous/steel/pipes" r:id="rId101"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" display="https://www.bigmint.co/prices/detail/erw-pipe-hr-coil-based-exy-delhi-india-1426-f-INR" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ22" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK22" display="https://www.bigmint.co/prices/ferrous/steel/pipes" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL22" display="https://www.bigmint.co/prices/detail/erw-pipe-hr-coil-based-exy-delhi-india-1426-f-INR" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ23" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ24" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AJ25" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK22" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AL22" display="https://www.bigmint.co/prices/ferrous/steel/pipes" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AM22" display="https://www.bigmint.co/prices/detail/erw-pipe-hr-coil-based-exy-delhi-india-1426-f-INR" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK23" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK24" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AK25" r:id="rId108"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11917,7 +11994,7 @@
         <v/>
       </c>
       <c r="AD2" s="41">
-        <f>Monthly!AH2-Monthly!AH12</f>
+        <f>Monthly!AI2-Monthly!AI12</f>
         <v/>
       </c>
     </row>
@@ -12040,7 +12117,7 @@
         <v/>
       </c>
       <c r="AD3" s="41">
-        <f>Monthly!AH2-Monthly!AH14</f>
+        <f>Monthly!AI2-Monthly!AI14</f>
         <v/>
       </c>
       <c r="AE3" s="20" t="n"/>
@@ -12164,7 +12241,7 @@
         <v/>
       </c>
       <c r="AD4" s="41">
-        <f>Monthly!AH2-Monthly!AH10</f>
+        <f>Monthly!AI2-Monthly!AI10</f>
         <v/>
       </c>
     </row>
@@ -12287,7 +12364,7 @@
         <v/>
       </c>
       <c r="AD5" s="42">
-        <f>Monthly!AH12-Monthly!AH14</f>
+        <f>Monthly!AI12-Monthly!AI14</f>
         <v/>
       </c>
     </row>
@@ -12410,7 +12487,7 @@
         <v/>
       </c>
       <c r="AD6" s="42">
-        <f>Monthly!AH12-Monthly!AH10</f>
+        <f>Monthly!AI12-Monthly!AI10</f>
         <v/>
       </c>
     </row>
@@ -12533,7 +12610,7 @@
         <v/>
       </c>
       <c r="AD7" s="42">
-        <f>Monthly!AH14-Monthly!AH10</f>
+        <f>Monthly!AI14-Monthly!AI10</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Track 14 more BigMint prices (HRC, GP, rebar by city)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/data/tracker.xlsx
+++ b/server/data/tracker.xlsx
@@ -1379,7 +1379,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1441,7 +1441,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1479,7 +1479,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -2060,7 +2060,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -2122,7 +2122,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -2160,7 +2160,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -2741,7 +2741,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -2803,7 +2803,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -2841,7 +2841,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -3422,7 +3422,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -3484,7 +3484,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -3522,7 +3522,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -4097,7 +4097,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -4159,7 +4159,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -4197,7 +4197,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -4778,7 +4778,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -4840,7 +4840,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -4878,7 +4878,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="en-US"/>
         </a:p>
@@ -5394,7 +5394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN25"/>
+  <dimension ref="A1:AN39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.6"/>
   <cols>
     <col width="51.5546875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8709,6 +8709,622 @@
       <c r="AK25" s="7" t="inlineStr">
         <is>
           <t>https://www.bigmint.co/prices/detail/ppgi-exy-mumbai-india-1369-f-INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>Hrc Exy Kolkata</t>
+        </is>
+      </c>
+      <c r="E26" s="1" t="n"/>
+      <c r="F26" s="1" t="n"/>
+      <c r="G26" s="1" t="n"/>
+      <c r="H26" s="1" t="n"/>
+      <c r="I26" s="1" t="n"/>
+      <c r="J26" s="1" t="n"/>
+      <c r="K26" s="1" t="n"/>
+      <c r="L26" s="1" t="n"/>
+      <c r="M26" s="1" t="n"/>
+      <c r="N26" s="1" t="n"/>
+      <c r="O26" s="1" t="n"/>
+      <c r="P26" s="1" t="n"/>
+      <c r="Q26" s="4" t="n"/>
+      <c r="R26" s="4" t="n"/>
+      <c r="S26" s="4" t="n"/>
+      <c r="T26" s="4" t="n"/>
+      <c r="U26" s="4" t="n"/>
+      <c r="V26" s="4" t="n"/>
+      <c r="W26" s="4" t="n"/>
+      <c r="X26" s="4" t="n"/>
+      <c r="Y26" s="4" t="n"/>
+      <c r="Z26" s="4" t="n"/>
+      <c r="AA26" s="4" t="n"/>
+      <c r="AB26" s="4" t="n"/>
+      <c r="AC26" s="4" t="n"/>
+      <c r="AD26" s="4" t="n"/>
+      <c r="AE26" s="4" t="n"/>
+      <c r="AF26" s="4" t="n"/>
+      <c r="AG26" s="4" t="n"/>
+      <c r="AH26" s="4" t="n"/>
+      <c r="AI26" s="4" t="n"/>
+      <c r="AJ26" s="9" t="n"/>
+      <c r="AK26" s="7" t="inlineStr">
+        <is>
+          <t>https://www.bigmint.co/prices/detail/hrc-exy-kolkata-india-1231-f-INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Hrc Exy Chennai</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="n"/>
+      <c r="F27" s="1" t="n"/>
+      <c r="G27" s="1" t="n"/>
+      <c r="H27" s="1" t="n"/>
+      <c r="I27" s="1" t="n"/>
+      <c r="J27" s="1" t="n"/>
+      <c r="K27" s="1" t="n"/>
+      <c r="L27" s="1" t="n"/>
+      <c r="M27" s="1" t="n"/>
+      <c r="N27" s="1" t="n"/>
+      <c r="O27" s="1" t="n"/>
+      <c r="P27" s="1" t="n"/>
+      <c r="Q27" s="4" t="n"/>
+      <c r="R27" s="4" t="n"/>
+      <c r="S27" s="4" t="n"/>
+      <c r="T27" s="4" t="n"/>
+      <c r="U27" s="4" t="n"/>
+      <c r="V27" s="4" t="n"/>
+      <c r="W27" s="4" t="n"/>
+      <c r="X27" s="4" t="n"/>
+      <c r="Y27" s="4" t="n"/>
+      <c r="Z27" s="4" t="n"/>
+      <c r="AA27" s="4" t="n"/>
+      <c r="AB27" s="4" t="n"/>
+      <c r="AC27" s="4" t="n"/>
+      <c r="AD27" s="4" t="n"/>
+      <c r="AE27" s="4" t="n"/>
+      <c r="AF27" s="4" t="n"/>
+      <c r="AG27" s="4" t="n"/>
+      <c r="AH27" s="4" t="n"/>
+      <c r="AI27" s="4" t="n"/>
+      <c r="AJ27" s="9" t="n"/>
+      <c r="AK27" s="7" t="inlineStr">
+        <is>
+          <t>https://www.bigmint.co/prices/detail/hrc-exy-chennai-india-1235-f-INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>Hrc Exy Hyderabad</t>
+        </is>
+      </c>
+      <c r="E28" s="1" t="n"/>
+      <c r="F28" s="1" t="n"/>
+      <c r="G28" s="1" t="n"/>
+      <c r="H28" s="1" t="n"/>
+      <c r="I28" s="1" t="n"/>
+      <c r="J28" s="1" t="n"/>
+      <c r="K28" s="1" t="n"/>
+      <c r="L28" s="1" t="n"/>
+      <c r="M28" s="1" t="n"/>
+      <c r="N28" s="1" t="n"/>
+      <c r="O28" s="1" t="n"/>
+      <c r="P28" s="1" t="n"/>
+      <c r="Q28" s="4" t="n"/>
+      <c r="R28" s="4" t="n"/>
+      <c r="S28" s="4" t="n"/>
+      <c r="T28" s="4" t="n"/>
+      <c r="U28" s="4" t="n"/>
+      <c r="V28" s="4" t="n"/>
+      <c r="W28" s="4" t="n"/>
+      <c r="X28" s="4" t="n"/>
+      <c r="Y28" s="4" t="n"/>
+      <c r="Z28" s="4" t="n"/>
+      <c r="AA28" s="4" t="n"/>
+      <c r="AB28" s="4" t="n"/>
+      <c r="AC28" s="4" t="n"/>
+      <c r="AD28" s="4" t="n"/>
+      <c r="AE28" s="4" t="n"/>
+      <c r="AF28" s="4" t="n"/>
+      <c r="AG28" s="4" t="n"/>
+      <c r="AH28" s="4" t="n"/>
+      <c r="AI28" s="4" t="n"/>
+      <c r="AJ28" s="9" t="n"/>
+      <c r="AK28" s="7" t="inlineStr">
+        <is>
+          <t>https://www.bigmint.co/prices/detail/hrc-exy-hyderabad-india-1236-f-INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>Hrc Exy Bangalore</t>
+        </is>
+      </c>
+      <c r="E29" s="1" t="n"/>
+      <c r="F29" s="1" t="n"/>
+      <c r="G29" s="1" t="n"/>
+      <c r="H29" s="1" t="n"/>
+      <c r="I29" s="1" t="n"/>
+      <c r="J29" s="1" t="n"/>
+      <c r="K29" s="1" t="n"/>
+      <c r="L29" s="1" t="n"/>
+      <c r="M29" s="1" t="n"/>
+      <c r="N29" s="1" t="n"/>
+      <c r="O29" s="1" t="n"/>
+      <c r="P29" s="1" t="n"/>
+      <c r="Q29" s="4" t="n"/>
+      <c r="R29" s="4" t="n"/>
+      <c r="S29" s="4" t="n"/>
+      <c r="T29" s="4" t="n"/>
+      <c r="U29" s="4" t="n"/>
+      <c r="V29" s="4" t="n"/>
+      <c r="W29" s="4" t="n"/>
+      <c r="X29" s="4" t="n"/>
+      <c r="Y29" s="4" t="n"/>
+      <c r="Z29" s="4" t="n"/>
+      <c r="AA29" s="4" t="n"/>
+      <c r="AB29" s="4" t="n"/>
+      <c r="AC29" s="4" t="n"/>
+      <c r="AD29" s="4" t="n"/>
+      <c r="AE29" s="4" t="n"/>
+      <c r="AF29" s="4" t="n"/>
+      <c r="AG29" s="4" t="n"/>
+      <c r="AH29" s="4" t="n"/>
+      <c r="AI29" s="4" t="n"/>
+      <c r="AJ29" s="9" t="n"/>
+      <c r="AK29" s="7" t="inlineStr">
+        <is>
+          <t>https://www.bigmint.co/prices/detail/hrc-exy-bangalore-india-1390-f-INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>Hrc Exy Faridabad</t>
+        </is>
+      </c>
+      <c r="E30" s="1" t="n"/>
+      <c r="F30" s="1" t="n"/>
+      <c r="G30" s="1" t="n"/>
+      <c r="H30" s="1" t="n"/>
+      <c r="I30" s="1" t="n"/>
+      <c r="J30" s="1" t="n"/>
+      <c r="K30" s="1" t="n"/>
+      <c r="L30" s="1" t="n"/>
+      <c r="M30" s="1" t="n"/>
+      <c r="N30" s="1" t="n"/>
+      <c r="O30" s="1" t="n"/>
+      <c r="P30" s="1" t="n"/>
+      <c r="Q30" s="4" t="n"/>
+      <c r="R30" s="4" t="n"/>
+      <c r="S30" s="4" t="n"/>
+      <c r="T30" s="4" t="n"/>
+      <c r="U30" s="4" t="n"/>
+      <c r="V30" s="4" t="n"/>
+      <c r="W30" s="4" t="n"/>
+      <c r="X30" s="4" t="n"/>
+      <c r="Y30" s="4" t="n"/>
+      <c r="Z30" s="4" t="n"/>
+      <c r="AA30" s="4" t="n"/>
+      <c r="AB30" s="4" t="n"/>
+      <c r="AC30" s="4" t="n"/>
+      <c r="AD30" s="4" t="n"/>
+      <c r="AE30" s="4" t="n"/>
+      <c r="AF30" s="4" t="n"/>
+      <c r="AG30" s="4" t="n"/>
+      <c r="AH30" s="4" t="n"/>
+      <c r="AI30" s="4" t="n"/>
+      <c r="AJ30" s="9" t="n"/>
+      <c r="AK30" s="7" t="inlineStr">
+        <is>
+          <t>https://www.bigmint.co/prices/detail/hrc-exy-faridabad-india-1229-f-INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>Hrc Exy Delhi</t>
+        </is>
+      </c>
+      <c r="E31" s="1" t="n"/>
+      <c r="F31" s="1" t="n"/>
+      <c r="G31" s="1" t="n"/>
+      <c r="H31" s="1" t="n"/>
+      <c r="I31" s="1" t="n"/>
+      <c r="J31" s="1" t="n"/>
+      <c r="K31" s="1" t="n"/>
+      <c r="L31" s="1" t="n"/>
+      <c r="M31" s="1" t="n"/>
+      <c r="N31" s="1" t="n"/>
+      <c r="O31" s="1" t="n"/>
+      <c r="P31" s="1" t="n"/>
+      <c r="Q31" s="4" t="n"/>
+      <c r="R31" s="4" t="n"/>
+      <c r="S31" s="4" t="n"/>
+      <c r="T31" s="4" t="n"/>
+      <c r="U31" s="4" t="n"/>
+      <c r="V31" s="4" t="n"/>
+      <c r="W31" s="4" t="n"/>
+      <c r="X31" s="4" t="n"/>
+      <c r="Y31" s="4" t="n"/>
+      <c r="Z31" s="4" t="n"/>
+      <c r="AA31" s="4" t="n"/>
+      <c r="AB31" s="4" t="n"/>
+      <c r="AC31" s="4" t="n"/>
+      <c r="AD31" s="4" t="n"/>
+      <c r="AE31" s="4" t="n"/>
+      <c r="AF31" s="4" t="n"/>
+      <c r="AG31" s="4" t="n"/>
+      <c r="AH31" s="4" t="n"/>
+      <c r="AI31" s="4" t="n"/>
+      <c r="AJ31" s="9" t="n"/>
+      <c r="AK31" s="7" t="inlineStr">
+        <is>
+          <t>https://www.bigmint.co/prices/detail/hrc-exy-delhi-india-1228-f-INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>Hrc Exy Ludhiana</t>
+        </is>
+      </c>
+      <c r="E32" s="1" t="n"/>
+      <c r="F32" s="1" t="n"/>
+      <c r="G32" s="1" t="n"/>
+      <c r="H32" s="1" t="n"/>
+      <c r="I32" s="1" t="n"/>
+      <c r="J32" s="1" t="n"/>
+      <c r="K32" s="1" t="n"/>
+      <c r="L32" s="1" t="n"/>
+      <c r="M32" s="1" t="n"/>
+      <c r="N32" s="1" t="n"/>
+      <c r="O32" s="1" t="n"/>
+      <c r="P32" s="1" t="n"/>
+      <c r="Q32" s="4" t="n"/>
+      <c r="R32" s="4" t="n"/>
+      <c r="S32" s="4" t="n"/>
+      <c r="T32" s="4" t="n"/>
+      <c r="U32" s="4" t="n"/>
+      <c r="V32" s="4" t="n"/>
+      <c r="W32" s="4" t="n"/>
+      <c r="X32" s="4" t="n"/>
+      <c r="Y32" s="4" t="n"/>
+      <c r="Z32" s="4" t="n"/>
+      <c r="AA32" s="4" t="n"/>
+      <c r="AB32" s="4" t="n"/>
+      <c r="AC32" s="4" t="n"/>
+      <c r="AD32" s="4" t="n"/>
+      <c r="AE32" s="4" t="n"/>
+      <c r="AF32" s="4" t="n"/>
+      <c r="AG32" s="4" t="n"/>
+      <c r="AH32" s="4" t="n"/>
+      <c r="AI32" s="4" t="n"/>
+      <c r="AJ32" s="9" t="n"/>
+      <c r="AK32" s="7" t="inlineStr">
+        <is>
+          <t>https://www.bigmint.co/prices/detail/hrc-exy-ludhiana-india-1230-f-INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>Hrc Exy Ahmedabad</t>
+        </is>
+      </c>
+      <c r="E33" s="1" t="n"/>
+      <c r="F33" s="1" t="n"/>
+      <c r="G33" s="1" t="n"/>
+      <c r="H33" s="1" t="n"/>
+      <c r="I33" s="1" t="n"/>
+      <c r="J33" s="1" t="n"/>
+      <c r="K33" s="1" t="n"/>
+      <c r="L33" s="1" t="n"/>
+      <c r="M33" s="1" t="n"/>
+      <c r="N33" s="1" t="n"/>
+      <c r="O33" s="1" t="n"/>
+      <c r="P33" s="1" t="n"/>
+      <c r="Q33" s="4" t="n"/>
+      <c r="R33" s="4" t="n"/>
+      <c r="S33" s="4" t="n"/>
+      <c r="T33" s="4" t="n"/>
+      <c r="U33" s="4" t="n"/>
+      <c r="V33" s="4" t="n"/>
+      <c r="W33" s="4" t="n"/>
+      <c r="X33" s="4" t="n"/>
+      <c r="Y33" s="4" t="n"/>
+      <c r="Z33" s="4" t="n"/>
+      <c r="AA33" s="4" t="n"/>
+      <c r="AB33" s="4" t="n"/>
+      <c r="AC33" s="4" t="n"/>
+      <c r="AD33" s="4" t="n"/>
+      <c r="AE33" s="4" t="n"/>
+      <c r="AF33" s="4" t="n"/>
+      <c r="AG33" s="4" t="n"/>
+      <c r="AH33" s="4" t="n"/>
+      <c r="AI33" s="4" t="n"/>
+      <c r="AJ33" s="9" t="n"/>
+      <c r="AK33" s="7" t="inlineStr">
+        <is>
+          <t>https://www.bigmint.co/prices/detail/hrc-exy-ahmedabad-india-1233-f-INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>Gp Exy Hyderabad</t>
+        </is>
+      </c>
+      <c r="E34" s="1" t="n"/>
+      <c r="F34" s="1" t="n"/>
+      <c r="G34" s="1" t="n"/>
+      <c r="H34" s="1" t="n"/>
+      <c r="I34" s="1" t="n"/>
+      <c r="J34" s="1" t="n"/>
+      <c r="K34" s="1" t="n"/>
+      <c r="L34" s="1" t="n"/>
+      <c r="M34" s="1" t="n"/>
+      <c r="N34" s="1" t="n"/>
+      <c r="O34" s="1" t="n"/>
+      <c r="P34" s="1" t="n"/>
+      <c r="Q34" s="4" t="n"/>
+      <c r="R34" s="4" t="n"/>
+      <c r="S34" s="4" t="n"/>
+      <c r="T34" s="4" t="n"/>
+      <c r="U34" s="4" t="n"/>
+      <c r="V34" s="4" t="n"/>
+      <c r="W34" s="4" t="n"/>
+      <c r="X34" s="4" t="n"/>
+      <c r="Y34" s="4" t="n"/>
+      <c r="Z34" s="4" t="n"/>
+      <c r="AA34" s="4" t="n"/>
+      <c r="AB34" s="4" t="n"/>
+      <c r="AC34" s="4" t="n"/>
+      <c r="AD34" s="4" t="n"/>
+      <c r="AE34" s="4" t="n"/>
+      <c r="AF34" s="4" t="n"/>
+      <c r="AG34" s="4" t="n"/>
+      <c r="AH34" s="4" t="n"/>
+      <c r="AI34" s="4" t="n"/>
+      <c r="AJ34" s="9" t="n"/>
+      <c r="AK34" s="7" t="inlineStr">
+        <is>
+          <t>https://www.bigmint.co/prices/detail/gp-exy-hyderabad-india-1679-f-INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>Gp Exy Chennai</t>
+        </is>
+      </c>
+      <c r="E35" s="1" t="n"/>
+      <c r="F35" s="1" t="n"/>
+      <c r="G35" s="1" t="n"/>
+      <c r="H35" s="1" t="n"/>
+      <c r="I35" s="1" t="n"/>
+      <c r="J35" s="1" t="n"/>
+      <c r="K35" s="1" t="n"/>
+      <c r="L35" s="1" t="n"/>
+      <c r="M35" s="1" t="n"/>
+      <c r="N35" s="1" t="n"/>
+      <c r="O35" s="1" t="n"/>
+      <c r="P35" s="1" t="n"/>
+      <c r="Q35" s="4" t="n"/>
+      <c r="R35" s="4" t="n"/>
+      <c r="S35" s="4" t="n"/>
+      <c r="T35" s="4" t="n"/>
+      <c r="U35" s="4" t="n"/>
+      <c r="V35" s="4" t="n"/>
+      <c r="W35" s="4" t="n"/>
+      <c r="X35" s="4" t="n"/>
+      <c r="Y35" s="4" t="n"/>
+      <c r="Z35" s="4" t="n"/>
+      <c r="AA35" s="4" t="n"/>
+      <c r="AB35" s="4" t="n"/>
+      <c r="AC35" s="4" t="n"/>
+      <c r="AD35" s="4" t="n"/>
+      <c r="AE35" s="4" t="n"/>
+      <c r="AF35" s="4" t="n"/>
+      <c r="AG35" s="4" t="n"/>
+      <c r="AH35" s="4" t="n"/>
+      <c r="AI35" s="4" t="n"/>
+      <c r="AJ35" s="9" t="n"/>
+      <c r="AK35" s="7" t="inlineStr">
+        <is>
+          <t>https://www.bigmint.co/prices/detail/gp-exy-chennai-india-1680-f-INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>Gp Exy Delhi</t>
+        </is>
+      </c>
+      <c r="E36" s="1" t="n"/>
+      <c r="F36" s="1" t="n"/>
+      <c r="G36" s="1" t="n"/>
+      <c r="H36" s="1" t="n"/>
+      <c r="I36" s="1" t="n"/>
+      <c r="J36" s="1" t="n"/>
+      <c r="K36" s="1" t="n"/>
+      <c r="L36" s="1" t="n"/>
+      <c r="M36" s="1" t="n"/>
+      <c r="N36" s="1" t="n"/>
+      <c r="O36" s="1" t="n"/>
+      <c r="P36" s="1" t="n"/>
+      <c r="Q36" s="4" t="n"/>
+      <c r="R36" s="4" t="n"/>
+      <c r="S36" s="4" t="n"/>
+      <c r="T36" s="4" t="n"/>
+      <c r="U36" s="4" t="n"/>
+      <c r="V36" s="4" t="n"/>
+      <c r="W36" s="4" t="n"/>
+      <c r="X36" s="4" t="n"/>
+      <c r="Y36" s="4" t="n"/>
+      <c r="Z36" s="4" t="n"/>
+      <c r="AA36" s="4" t="n"/>
+      <c r="AB36" s="4" t="n"/>
+      <c r="AC36" s="4" t="n"/>
+      <c r="AD36" s="4" t="n"/>
+      <c r="AE36" s="4" t="n"/>
+      <c r="AF36" s="4" t="n"/>
+      <c r="AG36" s="4" t="n"/>
+      <c r="AH36" s="4" t="n"/>
+      <c r="AI36" s="4" t="n"/>
+      <c r="AJ36" s="9" t="n"/>
+      <c r="AK36" s="7" t="inlineStr">
+        <is>
+          <t>https://www.bigmint.co/prices/detail/gp-exy-delhi-india-1681-f-INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>Rebar Exy Raipur</t>
+        </is>
+      </c>
+      <c r="E37" s="1" t="n"/>
+      <c r="F37" s="1" t="n"/>
+      <c r="G37" s="1" t="n"/>
+      <c r="H37" s="1" t="n"/>
+      <c r="I37" s="1" t="n"/>
+      <c r="J37" s="1" t="n"/>
+      <c r="K37" s="1" t="n"/>
+      <c r="L37" s="1" t="n"/>
+      <c r="M37" s="1" t="n"/>
+      <c r="N37" s="1" t="n"/>
+      <c r="O37" s="1" t="n"/>
+      <c r="P37" s="1" t="n"/>
+      <c r="Q37" s="4" t="n"/>
+      <c r="R37" s="4" t="n"/>
+      <c r="S37" s="4" t="n"/>
+      <c r="T37" s="4" t="n"/>
+      <c r="U37" s="4" t="n"/>
+      <c r="V37" s="4" t="n"/>
+      <c r="W37" s="4" t="n"/>
+      <c r="X37" s="4" t="n"/>
+      <c r="Y37" s="4" t="n"/>
+      <c r="Z37" s="4" t="n"/>
+      <c r="AA37" s="4" t="n"/>
+      <c r="AB37" s="4" t="n"/>
+      <c r="AC37" s="4" t="n"/>
+      <c r="AD37" s="4" t="n"/>
+      <c r="AE37" s="4" t="n"/>
+      <c r="AF37" s="4" t="n"/>
+      <c r="AG37" s="4" t="n"/>
+      <c r="AH37" s="4" t="n"/>
+      <c r="AI37" s="4" t="n"/>
+      <c r="AJ37" s="9" t="n"/>
+      <c r="AK37" s="7" t="inlineStr">
+        <is>
+          <t>https://www.bigmint.co/prices/detail/rebar-exy-raipur-india-1922-f-INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>Rebar Exw Raipur</t>
+        </is>
+      </c>
+      <c r="E38" s="1" t="n"/>
+      <c r="F38" s="1" t="n"/>
+      <c r="G38" s="1" t="n"/>
+      <c r="H38" s="1" t="n"/>
+      <c r="I38" s="1" t="n"/>
+      <c r="J38" s="1" t="n"/>
+      <c r="K38" s="1" t="n"/>
+      <c r="L38" s="1" t="n"/>
+      <c r="M38" s="1" t="n"/>
+      <c r="N38" s="1" t="n"/>
+      <c r="O38" s="1" t="n"/>
+      <c r="P38" s="1" t="n"/>
+      <c r="Q38" s="4" t="n"/>
+      <c r="R38" s="4" t="n"/>
+      <c r="S38" s="4" t="n"/>
+      <c r="T38" s="4" t="n"/>
+      <c r="U38" s="4" t="n"/>
+      <c r="V38" s="4" t="n"/>
+      <c r="W38" s="4" t="n"/>
+      <c r="X38" s="4" t="n"/>
+      <c r="Y38" s="4" t="n"/>
+      <c r="Z38" s="4" t="n"/>
+      <c r="AA38" s="4" t="n"/>
+      <c r="AB38" s="4" t="n"/>
+      <c r="AC38" s="4" t="n"/>
+      <c r="AD38" s="4" t="n"/>
+      <c r="AE38" s="4" t="n"/>
+      <c r="AF38" s="4" t="n"/>
+      <c r="AG38" s="4" t="n"/>
+      <c r="AH38" s="4" t="n"/>
+      <c r="AI38" s="4" t="n"/>
+      <c r="AJ38" s="9" t="n"/>
+      <c r="AK38" s="7" t="inlineStr">
+        <is>
+          <t>https://www.bigmint.co/prices/detail/rebar-exw-raipur-india-1503-f-INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>Rebar Exw Jalna</t>
+        </is>
+      </c>
+      <c r="E39" s="1" t="n"/>
+      <c r="F39" s="1" t="n"/>
+      <c r="G39" s="1" t="n"/>
+      <c r="H39" s="1" t="n"/>
+      <c r="I39" s="1" t="n"/>
+      <c r="J39" s="1" t="n"/>
+      <c r="K39" s="1" t="n"/>
+      <c r="L39" s="1" t="n"/>
+      <c r="M39" s="1" t="n"/>
+      <c r="N39" s="1" t="n"/>
+      <c r="O39" s="1" t="n"/>
+      <c r="P39" s="1" t="n"/>
+      <c r="Q39" s="4" t="n"/>
+      <c r="R39" s="4" t="n"/>
+      <c r="S39" s="4" t="n"/>
+      <c r="T39" s="4" t="n"/>
+      <c r="U39" s="4" t="n"/>
+      <c r="V39" s="4" t="n"/>
+      <c r="W39" s="4" t="n"/>
+      <c r="X39" s="4" t="n"/>
+      <c r="Y39" s="4" t="n"/>
+      <c r="Z39" s="4" t="n"/>
+      <c r="AA39" s="4" t="n"/>
+      <c r="AB39" s="4" t="n"/>
+      <c r="AC39" s="4" t="n"/>
+      <c r="AD39" s="4" t="n"/>
+      <c r="AE39" s="4" t="n"/>
+      <c r="AF39" s="4" t="n"/>
+      <c r="AG39" s="4" t="n"/>
+      <c r="AH39" s="4" t="n"/>
+      <c r="AI39" s="4" t="n"/>
+      <c r="AJ39" s="9" t="n"/>
+      <c r="AK39" s="7" t="inlineStr">
+        <is>
+          <t>https://www.bigmint.co/prices/detail/rebar-exw-jalna-india-1121-f-INR</t>
         </is>
       </c>
     </row>

</xml_diff>